<commit_message>
save before trying new coding rules
</commit_message>
<xml_diff>
--- a/Austerlitz/Turns/124TMay1812.xlsx
+++ b/Austerlitz/Turns/124TMay1812.xlsx
@@ -162,9 +162,6 @@
   </x:si>
   <x:si>
     <x:t>State</x:t>
-  </x:si>
-  <x:si>
-    <x:t>-</x:t>
   </x:si>
   <x:si>
     <x:t>(17) Trade and Loading - 1 (Goods/Quantity/Source/Destination)</x:t>
@@ -946,7 +943,7 @@
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
   <x:dimension ref="A1:L308"/>
-  <x:sheetFormatPr defaultColWidth="10.710625" defaultRowHeight="15" customHeight="1"/>
+  <x:sheetFormatPr defaultColWidth="10.599514" defaultRowHeight="15" customHeight="1"/>
   <x:cols>
     <x:col min="1" max="1" width="3.570312" style="0" customWidth="1"/>
     <x:col min="2" max="6" width="7.140625" style="0" customWidth="1"/>
@@ -1133,13 +1130,25 @@
       <x:c r="A12" s="4">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B12" s="45"/>
-      <x:c r="C12" s="45"/>
-      <x:c r="D12" s="46"/>
-      <x:c r="E12" s="45"/>
-      <x:c r="F12" s="45"/>
+      <x:c r="B12" s="45">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C12" s="45">
+        <x:v>273</x:v>
+      </x:c>
+      <x:c r="D12" s="46">
+        <x:v>13483250</x:v>
+      </x:c>
+      <x:c r="E12" s="45">
+        <x:v>82590</x:v>
+      </x:c>
+      <x:c r="F12" s="45">
+        <x:v>23452</x:v>
+      </x:c>
       <x:c r="G12" s="45"/>
-      <x:c r="H12" s="45"/>
+      <x:c r="H12" s="45">
+        <x:v>34849</x:v>
+      </x:c>
       <x:c r="I12" s="45"/>
       <x:c r="K12" s="5"/>
       <x:c r="L12" s="5">
@@ -1192,11 +1201,21 @@
       <x:c r="A13" s="4">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B13" s="45"/>
-      <x:c r="C13" s="45"/>
-      <x:c r="D13" s="45"/>
-      <x:c r="E13" s="45"/>
-      <x:c r="F13" s="45"/>
+      <x:c r="B13" s="45">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C13" s="45">
+        <x:v>274</x:v>
+      </x:c>
+      <x:c r="D13" s="45">
+        <x:v>68560</x:v>
+      </x:c>
+      <x:c r="E13" s="45">
+        <x:v>792</x:v>
+      </x:c>
+      <x:c r="F13" s="45">
+        <x:v>259</x:v>
+      </x:c>
       <x:c r="G13" s="45"/>
       <x:c r="H13" s="45"/>
       <x:c r="I13" s="45"/>
@@ -1251,11 +1270,19 @@
       <x:c r="A14" s="4">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B14" s="45"/>
-      <x:c r="C14" s="45"/>
-      <x:c r="D14" s="45"/>
+      <x:c r="B14" s="45">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C14" s="45">
+        <x:v>273</x:v>
+      </x:c>
+      <x:c r="D14" s="45">
+        <x:v>912800</x:v>
+      </x:c>
       <x:c r="E14" s="45"/>
-      <x:c r="F14" s="45"/>
+      <x:c r="F14" s="45">
+        <x:v>1788</x:v>
+      </x:c>
       <x:c r="G14" s="45"/>
       <x:c r="H14" s="45"/>
       <x:c r="I14" s="45"/>
@@ -1310,13 +1337,25 @@
       <x:c r="A15" s="4">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B15" s="45"/>
-      <x:c r="C15" s="45"/>
-      <x:c r="D15" s="45"/>
-      <x:c r="E15" s="45"/>
-      <x:c r="F15" s="45"/>
+      <x:c r="B15" s="45">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C15" s="45">
+        <x:v>273</x:v>
+      </x:c>
+      <x:c r="D15" s="45">
+        <x:v>13483250</x:v>
+      </x:c>
+      <x:c r="E15" s="45">
+        <x:v>82590</x:v>
+      </x:c>
+      <x:c r="F15" s="45">
+        <x:v>23452</x:v>
+      </x:c>
       <x:c r="G15" s="45"/>
-      <x:c r="H15" s="45"/>
+      <x:c r="H15" s="45">
+        <x:v>34849</x:v>
+      </x:c>
       <x:c r="I15" s="45"/>
       <x:c r="K15" s="5"/>
       <x:c r="L15" s="5">
@@ -1369,13 +1408,25 @@
       <x:c r="A16" s="4">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B16" s="45"/>
-      <x:c r="C16" s="45"/>
-      <x:c r="D16" s="45"/>
-      <x:c r="E16" s="45"/>
-      <x:c r="F16" s="45"/>
+      <x:c r="B16" s="45">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C16" s="45">
+        <x:v>274</x:v>
+      </x:c>
+      <x:c r="D16" s="45">
+        <x:v>1233565</x:v>
+      </x:c>
+      <x:c r="E16" s="45">
+        <x:v>15577</x:v>
+      </x:c>
+      <x:c r="F16" s="45">
+        <x:v>1932</x:v>
+      </x:c>
       <x:c r="G16" s="45"/>
-      <x:c r="H16" s="45"/>
+      <x:c r="H16" s="45">
+        <x:v>276</x:v>
+      </x:c>
       <x:c r="I16" s="45"/>
       <x:c r="K16" s="5"/>
       <x:c r="L16" s="5">
@@ -1428,11 +1479,19 @@
       <x:c r="A17" s="4">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B17" s="45"/>
-      <x:c r="C17" s="45"/>
-      <x:c r="D17" s="45"/>
+      <x:c r="B17" s="45">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C17" s="45">
+        <x:v>273</x:v>
+      </x:c>
+      <x:c r="D17" s="45">
+        <x:v>912800</x:v>
+      </x:c>
       <x:c r="E17" s="45"/>
-      <x:c r="F17" s="45"/>
+      <x:c r="F17" s="45">
+        <x:v>1788</x:v>
+      </x:c>
       <x:c r="G17" s="45"/>
       <x:c r="H17" s="45"/>
       <x:c r="I17" s="45"/>
@@ -1487,11 +1546,19 @@
       <x:c r="A18" s="4">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B18" s="45"/>
-      <x:c r="C18" s="45"/>
-      <x:c r="D18" s="45"/>
+      <x:c r="B18" s="45">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C18" s="45">
+        <x:v>274</x:v>
+      </x:c>
+      <x:c r="D18" s="45">
+        <x:v>826400</x:v>
+      </x:c>
       <x:c r="E18" s="45"/>
-      <x:c r="F18" s="45"/>
+      <x:c r="F18" s="45">
+        <x:v>1584</x:v>
+      </x:c>
       <x:c r="G18" s="45"/>
       <x:c r="H18" s="45"/>
       <x:c r="I18" s="45"/>
@@ -2741,8 +2808,12 @@
       <x:c r="A54" s="4">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B54" s="49"/>
-      <x:c r="C54" s="45"/>
+      <x:c r="B54" s="49">
+        <x:v>4072</x:v>
+      </x:c>
+      <x:c r="C54" s="45">
+        <x:v>800</x:v>
+      </x:c>
       <x:c r="D54" s="4"/>
       <x:c r="E54" s="4"/>
       <x:c r="F54" s="4"/>
@@ -2777,8 +2848,12 @@
       <x:c r="A55" s="4">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B55" s="49"/>
-      <x:c r="C55" s="45"/>
+      <x:c r="B55" s="49">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="C55" s="45">
+        <x:v>800</x:v>
+      </x:c>
       <x:c r="D55" s="4"/>
       <x:c r="E55" s="4"/>
       <x:c r="F55" s="4"/>
@@ -2813,8 +2888,12 @@
       <x:c r="A56" s="4">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B56" s="49"/>
-      <x:c r="C56" s="49"/>
+      <x:c r="B56" s="49">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="C56" s="49">
+        <x:v>800</x:v>
+      </x:c>
       <x:c r="D56" s="4"/>
       <x:c r="E56" s="4"/>
       <x:c r="F56" s="4"/>
@@ -2849,8 +2928,12 @@
       <x:c r="A57" s="4">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B57" s="45"/>
-      <x:c r="C57" s="45"/>
+      <x:c r="B57" s="45">
+        <x:v>79</x:v>
+      </x:c>
+      <x:c r="C57" s="45">
+        <x:v>800</x:v>
+      </x:c>
       <x:c r="D57" s="4"/>
       <x:c r="E57" s="4"/>
       <x:c r="F57" s="4"/>
@@ -3217,7 +3300,9 @@
       <x:c r="A69" s="4">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B69" s="45"/>
+      <x:c r="B69" s="45">
+        <x:v>61</x:v>
+      </x:c>
       <x:c r="C69" s="4"/>
       <x:c r="D69" s="4"/>
       <x:c r="E69" s="4"/>
@@ -3244,7 +3329,9 @@
       <x:c r="A70" s="4">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B70" s="45"/>
+      <x:c r="B70" s="45">
+        <x:v>4079</x:v>
+      </x:c>
       <x:c r="C70" s="4"/>
       <x:c r="D70" s="4"/>
       <x:c r="E70" s="4"/>
@@ -3271,7 +3358,9 @@
       <x:c r="A71" s="4">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B71" s="45"/>
+      <x:c r="B71" s="45">
+        <x:v>79</x:v>
+      </x:c>
       <x:c r="C71" s="4"/>
       <x:c r="D71" s="4"/>
       <x:c r="E71" s="4"/>
@@ -3298,7 +3387,9 @@
       <x:c r="A72" s="4">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B72" s="45"/>
+      <x:c r="B72" s="45">
+        <x:v>77</x:v>
+      </x:c>
       <x:c r="C72" s="4"/>
       <x:c r="D72" s="4"/>
       <x:c r="E72" s="4"/>
@@ -5286,9 +5377,15 @@
       <x:c r="A143" s="4">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B143" s="45"/>
-      <x:c r="C143" s="45"/>
-      <x:c r="D143" s="45"/>
+      <x:c r="B143" s="45">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C143" s="45">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="D143" s="45">
+        <x:v>27</x:v>
+      </x:c>
       <x:c r="E143" s="4"/>
       <x:c r="F143" s="4"/>
       <x:c r="G143" s="4"/>
@@ -5326,9 +5423,15 @@
       <x:c r="A144" s="4">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B144" s="45"/>
-      <x:c r="C144" s="45"/>
-      <x:c r="D144" s="45"/>
+      <x:c r="B144" s="45">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C144" s="45">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="D144" s="45">
+        <x:v>65</x:v>
+      </x:c>
       <x:c r="E144" s="4"/>
       <x:c r="F144" s="4"/>
       <x:c r="G144" s="4"/>
@@ -5366,9 +5469,15 @@
       <x:c r="A145" s="4">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B145" s="49"/>
-      <x:c r="C145" s="45"/>
-      <x:c r="D145" s="45"/>
+      <x:c r="B145" s="49">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C145" s="45">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="D145" s="45">
+        <x:v>61</x:v>
+      </x:c>
       <x:c r="E145" s="4"/>
       <x:c r="F145" s="4"/>
       <x:c r="G145" s="4"/>
@@ -5406,9 +5515,15 @@
       <x:c r="A146" s="4">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B146" s="49"/>
-      <x:c r="C146" s="45"/>
-      <x:c r="D146" s="49"/>
+      <x:c r="B146" s="49">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C146" s="45">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="D146" s="49">
+        <x:v>64</x:v>
+      </x:c>
       <x:c r="E146" s="4"/>
       <x:c r="F146" s="4"/>
       <x:c r="G146" s="4"/>
@@ -5730,8 +5845,12 @@
       <x:c r="A156" s="4">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B156" s="45"/>
-      <x:c r="C156" s="45"/>
+      <x:c r="B156" s="45">
+        <x:v>4095</x:v>
+      </x:c>
+      <x:c r="C156" s="45">
+        <x:v>65</x:v>
+      </x:c>
       <x:c r="D156" s="4"/>
       <x:c r="E156" s="4"/>
       <x:c r="F156" s="4"/>
@@ -5787,8 +5906,12 @@
       <x:c r="A157" s="4">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B157" s="45"/>
-      <x:c r="C157" s="45"/>
+      <x:c r="B157" s="45">
+        <x:v>4824</x:v>
+      </x:c>
+      <x:c r="C157" s="45">
+        <x:v>65</x:v>
+      </x:c>
       <x:c r="D157" s="4"/>
       <x:c r="E157" s="4"/>
       <x:c r="F157" s="4"/>
@@ -5844,8 +5967,12 @@
       <x:c r="A158" s="4">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B158" s="45"/>
-      <x:c r="C158" s="45"/>
+      <x:c r="B158" s="45">
+        <x:v>5031</x:v>
+      </x:c>
+      <x:c r="C158" s="45">
+        <x:v>65</x:v>
+      </x:c>
       <x:c r="D158" s="4"/>
       <x:c r="E158" s="4"/>
       <x:c r="F158" s="4"/>
@@ -5901,8 +6028,12 @@
       <x:c r="A159" s="4">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B159" s="45"/>
-      <x:c r="C159" s="45"/>
+      <x:c r="B159" s="45">
+        <x:v>5090</x:v>
+      </x:c>
+      <x:c r="C159" s="45">
+        <x:v>65</x:v>
+      </x:c>
       <x:c r="D159" s="4"/>
       <x:c r="E159" s="4"/>
       <x:c r="F159" s="4"/>
@@ -5958,8 +6089,12 @@
       <x:c r="A160" s="4">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B160" s="45"/>
-      <x:c r="C160" s="45"/>
+      <x:c r="B160" s="45">
+        <x:v>5167</x:v>
+      </x:c>
+      <x:c r="C160" s="45">
+        <x:v>65</x:v>
+      </x:c>
       <x:c r="D160" s="4"/>
       <x:c r="E160" s="4"/>
       <x:c r="F160" s="4"/>
@@ -6015,8 +6150,12 @@
       <x:c r="A161" s="4">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B161" s="45"/>
-      <x:c r="C161" s="45"/>
+      <x:c r="B161" s="45">
+        <x:v>5877</x:v>
+      </x:c>
+      <x:c r="C161" s="45">
+        <x:v>65</x:v>
+      </x:c>
       <x:c r="D161" s="4"/>
       <x:c r="E161" s="4"/>
       <x:c r="F161" s="4"/>
@@ -6072,8 +6211,12 @@
       <x:c r="A162" s="4">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B162" s="45"/>
-      <x:c r="C162" s="45"/>
+      <x:c r="B162" s="45">
+        <x:v>5880</x:v>
+      </x:c>
+      <x:c r="C162" s="45">
+        <x:v>65</x:v>
+      </x:c>
       <x:c r="D162" s="4"/>
       <x:c r="E162" s="4"/>
       <x:c r="F162" s="4"/>
@@ -6129,8 +6272,12 @@
       <x:c r="A163" s="4">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B163" s="45"/>
-      <x:c r="C163" s="45"/>
+      <x:c r="B163" s="45">
+        <x:v>5883</x:v>
+      </x:c>
+      <x:c r="C163" s="45">
+        <x:v>65</x:v>
+      </x:c>
       <x:c r="D163" s="4"/>
       <x:c r="E163" s="4"/>
       <x:c r="F163" s="4"/>
@@ -6186,8 +6333,12 @@
       <x:c r="A164" s="4">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="B164" s="45"/>
-      <x:c r="C164" s="45"/>
+      <x:c r="B164" s="45">
+        <x:v>4080</x:v>
+      </x:c>
+      <x:c r="C164" s="45">
+        <x:v>80</x:v>
+      </x:c>
       <x:c r="D164" s="4"/>
       <x:c r="E164" s="22"/>
       <x:c r="F164" s="22"/>
@@ -6243,8 +6394,12 @@
       <x:c r="A165" s="4">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="B165" s="45"/>
-      <x:c r="C165" s="45"/>
+      <x:c r="B165" s="45">
+        <x:v>4079</x:v>
+      </x:c>
+      <x:c r="C165" s="45">
+        <x:v>80</x:v>
+      </x:c>
       <x:c r="D165" s="4"/>
       <x:c r="E165" s="22"/>
       <x:c r="F165" s="22"/>
@@ -6300,8 +6455,12 @@
       <x:c r="A166" s="4">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="B166" s="49"/>
-      <x:c r="C166" s="45"/>
+      <x:c r="B166" s="49">
+        <x:v>5794</x:v>
+      </x:c>
+      <x:c r="C166" s="45">
+        <x:v>80</x:v>
+      </x:c>
       <x:c r="D166" s="4"/>
       <x:c r="E166" s="22"/>
       <x:c r="F166" s="22"/>
@@ -6357,8 +6516,12 @@
       <x:c r="A167" s="4">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="B167" s="45"/>
-      <x:c r="C167" s="49"/>
+      <x:c r="B167" s="45">
+        <x:v>5787</x:v>
+      </x:c>
+      <x:c r="C167" s="49">
+        <x:v>80</x:v>
+      </x:c>
       <x:c r="D167" s="4"/>
       <x:c r="E167" s="22"/>
       <x:c r="F167" s="22"/>
@@ -6414,8 +6577,12 @@
       <x:c r="A168" s="4">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="B168" s="45"/>
-      <x:c r="C168" s="45"/>
+      <x:c r="B168" s="45">
+        <x:v>5780</x:v>
+      </x:c>
+      <x:c r="C168" s="45">
+        <x:v>80</x:v>
+      </x:c>
       <x:c r="D168" s="4"/>
       <x:c r="E168" s="22"/>
       <x:c r="F168" s="22"/>
@@ -6471,8 +6638,12 @@
       <x:c r="A169" s="4">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="B169" s="45"/>
-      <x:c r="C169" s="45"/>
+      <x:c r="B169" s="45">
+        <x:v>5733</x:v>
+      </x:c>
+      <x:c r="C169" s="45">
+        <x:v>80</x:v>
+      </x:c>
       <x:c r="D169" s="4"/>
       <x:c r="E169" s="22"/>
       <x:c r="F169" s="22"/>
@@ -6528,8 +6699,12 @@
       <x:c r="A170" s="4">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="B170" s="45"/>
-      <x:c r="C170" s="45"/>
+      <x:c r="B170" s="45">
+        <x:v>5725</x:v>
+      </x:c>
+      <x:c r="C170" s="45">
+        <x:v>80</x:v>
+      </x:c>
       <x:c r="D170" s="4"/>
       <x:c r="E170" s="22"/>
       <x:c r="F170" s="22"/>
@@ -6585,8 +6760,12 @@
       <x:c r="A171" s="4">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="B171" s="45"/>
-      <x:c r="C171" s="45"/>
+      <x:c r="B171" s="45">
+        <x:v>5723</x:v>
+      </x:c>
+      <x:c r="C171" s="45">
+        <x:v>80</x:v>
+      </x:c>
       <x:c r="D171" s="4"/>
       <x:c r="E171" s="22"/>
       <x:c r="F171" s="22"/>
@@ -6642,8 +6821,12 @@
       <x:c r="A172" s="4">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="B172" s="45"/>
-      <x:c r="C172" s="45"/>
+      <x:c r="B172" s="45">
+        <x:v>5628</x:v>
+      </x:c>
+      <x:c r="C172" s="45">
+        <x:v>80</x:v>
+      </x:c>
       <x:c r="D172" s="4"/>
       <x:c r="E172" s="22"/>
       <x:c r="F172" s="22"/>
@@ -6699,8 +6882,12 @@
       <x:c r="A173" s="4">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="B173" s="45"/>
-      <x:c r="C173" s="45"/>
+      <x:c r="B173" s="45">
+        <x:v>5622</x:v>
+      </x:c>
+      <x:c r="C173" s="45">
+        <x:v>80</x:v>
+      </x:c>
       <x:c r="D173" s="4"/>
       <x:c r="E173" s="22"/>
       <x:c r="F173" s="22"/>
@@ -6756,8 +6943,12 @@
       <x:c r="A174" s="4">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="B174" s="45"/>
-      <x:c r="C174" s="45"/>
+      <x:c r="B174" s="45">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C174" s="45">
+        <x:v>80</x:v>
+      </x:c>
       <x:c r="D174" s="4"/>
       <x:c r="E174" s="22"/>
       <x:c r="F174" s="22"/>
@@ -7143,21 +7334,11 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B188" s="49"/>
-      <x:c r="C188" s="49" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="D188" s="49" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="E188" s="49" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="F188" s="49" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="G188" s="49" t="s">
-        <x:v>49</x:v>
-      </x:c>
+      <x:c r="C188" s="49"/>
+      <x:c r="D188" s="49"/>
+      <x:c r="E188" s="49"/>
+      <x:c r="F188" s="49"/>
+      <x:c r="G188" s="49"/>
       <x:c r="H188" s="4"/>
       <x:c r="I188" s="4"/>
       <x:c r="J188" s="4"/>
@@ -7181,21 +7362,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B189" s="49"/>
-      <x:c r="C189" s="49" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="D189" s="49" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="E189" s="49" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="F189" s="49" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="G189" s="49" t="s">
-        <x:v>49</x:v>
-      </x:c>
+      <x:c r="C189" s="49"/>
+      <x:c r="D189" s="49"/>
+      <x:c r="E189" s="49"/>
+      <x:c r="F189" s="49"/>
+      <x:c r="G189" s="49"/>
       <x:c r="H189" s="4"/>
       <x:c r="I189" s="4"/>
       <x:c r="J189" s="4"/>
@@ -7219,21 +7390,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B190" s="45"/>
-      <x:c r="C190" s="49" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="D190" s="49" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="E190" s="49" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="F190" s="49" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="G190" s="49" t="s">
-        <x:v>49</x:v>
-      </x:c>
+      <x:c r="C190" s="49"/>
+      <x:c r="D190" s="49"/>
+      <x:c r="E190" s="49"/>
+      <x:c r="F190" s="49"/>
+      <x:c r="G190" s="49"/>
       <x:c r="H190" s="4"/>
       <x:c r="I190" s="4"/>
       <x:c r="J190" s="4"/>
@@ -7268,7 +7429,7 @@
     </x:row>
     <x:row r="192" spans="1:12" ht="13.5" customHeight="1">
       <x:c r="A192" s="43" t="s">
-        <x:v>50</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="B192" s="4"/>
       <x:c r="C192" s="4"/>
@@ -7285,16 +7446,16 @@
     <x:row r="193" spans="1:12" ht="13.5" customHeight="1">
       <x:c r="A193" s="4"/>
       <x:c r="B193" s="4" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="C193" s="4" t="s">
         <x:v>51</x:v>
       </x:c>
-      <x:c r="C193" s="4" t="s">
+      <x:c r="D193" s="4" t="s">
         <x:v>52</x:v>
       </x:c>
-      <x:c r="D193" s="4" t="s">
+      <x:c r="E193" s="4" t="s">
         <x:v>53</x:v>
-      </x:c>
-      <x:c r="E193" s="4" t="s">
-        <x:v>54</x:v>
       </x:c>
       <x:c r="F193" s="4"/>
       <x:c r="G193" s="4"/>
@@ -8562,7 +8723,7 @@
     </x:row>
     <x:row r="213" spans="1:12" ht="13.5" customHeight="1">
       <x:c r="A213" s="43" t="s">
-        <x:v>55</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="B213" s="4"/>
       <x:c r="C213" s="4"/>
@@ -8579,25 +8740,25 @@
     <x:row r="214" spans="1:12" ht="13.5" customHeight="1">
       <x:c r="A214" s="4"/>
       <x:c r="B214" s="4" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="C214" s="4" t="s">
         <x:v>56</x:v>
       </x:c>
-      <x:c r="C214" s="4" t="s">
+      <x:c r="D214" s="4" t="s">
         <x:v>57</x:v>
       </x:c>
-      <x:c r="D214" s="4" t="s">
+      <x:c r="E214" s="4" t="s">
         <x:v>58</x:v>
       </x:c>
-      <x:c r="E214" s="4" t="s">
+      <x:c r="F214" s="4" t="s">
         <x:v>59</x:v>
       </x:c>
-      <x:c r="F214" s="4" t="s">
+      <x:c r="G214" s="4" t="s">
         <x:v>60</x:v>
       </x:c>
-      <x:c r="G214" s="4" t="s">
+      <x:c r="H214" s="4" t="s">
         <x:v>61</x:v>
-      </x:c>
-      <x:c r="H214" s="4" t="s">
-        <x:v>62</x:v>
       </x:c>
       <x:c r="I214" s="4"/>
       <x:c r="J214" s="4"/>
@@ -8609,12 +8770,20 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B215" s="49">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="C215" s="45">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D215" s="45">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E215" s="45">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="C215" s="45"/>
-      <x:c r="D215" s="45"/>
-      <x:c r="E215" s="45"/>
-      <x:c r="F215" s="45"/>
+      <x:c r="F215" s="45">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="G215" s="45"/>
       <x:c r="H215" s="45"/>
       <x:c r="I215" s="4"/>
@@ -8674,14 +8843,26 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B216" s="45">
-        <x:v>5320</x:v>
-      </x:c>
-      <x:c r="C216" s="45"/>
-      <x:c r="D216" s="45"/>
-      <x:c r="E216" s="45"/>
-      <x:c r="F216" s="45"/>
-      <x:c r="G216" s="45"/>
-      <x:c r="H216" s="45"/>
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="C216" s="45">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D216" s="45">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E216" s="45">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F216" s="45">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G216" s="45">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H216" s="45">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="I216" s="4"/>
       <x:c r="J216" s="4"/>
       <x:c r="K216" s="5"/>
@@ -8739,12 +8920,20 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B217" s="45">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="C217" s="45"/>
-      <x:c r="D217" s="45"/>
-      <x:c r="E217" s="45"/>
-      <x:c r="F217" s="45"/>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C217" s="45">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D217" s="45">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E217" s="45">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F217" s="45">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="G217" s="45"/>
       <x:c r="H217" s="45"/>
       <x:c r="I217" s="4"/>
@@ -8803,13 +8992,27 @@
       <x:c r="A218" s="4">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B218" s="45"/>
-      <x:c r="C218" s="45"/>
-      <x:c r="D218" s="45"/>
-      <x:c r="E218" s="45"/>
-      <x:c r="F218" s="45"/>
-      <x:c r="G218" s="45"/>
-      <x:c r="H218" s="45"/>
+      <x:c r="B218" s="45">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C218" s="45">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D218" s="45">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E218" s="45">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F218" s="45">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="G218" s="45">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H218" s="45">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="I218" s="4"/>
       <x:c r="J218" s="4"/>
       <x:c r="K218" s="5"/>
@@ -8866,11 +9069,21 @@
       <x:c r="A219" s="4">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B219" s="45"/>
-      <x:c r="C219" s="45"/>
-      <x:c r="D219" s="45"/>
-      <x:c r="E219" s="45"/>
-      <x:c r="F219" s="45"/>
+      <x:c r="B219" s="45">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C219" s="45">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D219" s="45">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E219" s="45">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F219" s="45">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="G219" s="45"/>
       <x:c r="H219" s="45"/>
       <x:c r="I219" s="4"/>
@@ -8929,13 +9142,27 @@
       <x:c r="A220" s="4">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B220" s="45"/>
-      <x:c r="C220" s="45"/>
-      <x:c r="D220" s="45"/>
-      <x:c r="E220" s="45"/>
-      <x:c r="F220" s="45"/>
-      <x:c r="G220" s="45"/>
-      <x:c r="H220" s="45"/>
+      <x:c r="B220" s="45">
+        <x:v>79</x:v>
+      </x:c>
+      <x:c r="C220" s="45">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D220" s="45">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E220" s="45">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F220" s="45">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G220" s="45">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H220" s="45">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="I220" s="4"/>
       <x:c r="J220" s="4"/>
       <x:c r="K220" s="5"/>
@@ -8992,11 +9219,21 @@
       <x:c r="A221" s="4">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B221" s="45"/>
-      <x:c r="C221" s="45"/>
-      <x:c r="D221" s="45"/>
-      <x:c r="E221" s="45"/>
-      <x:c r="F221" s="45"/>
+      <x:c r="B221" s="45">
+        <x:v>4447</x:v>
+      </x:c>
+      <x:c r="C221" s="45">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D221" s="45">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E221" s="45">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F221" s="45">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="G221" s="45"/>
       <x:c r="H221" s="45"/>
       <x:c r="I221" s="4"/>
@@ -9055,11 +9292,21 @@
       <x:c r="A222" s="4">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B222" s="45"/>
-      <x:c r="C222" s="45"/>
-      <x:c r="D222" s="45"/>
-      <x:c r="E222" s="45"/>
-      <x:c r="F222" s="45"/>
+      <x:c r="B222" s="45">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="C222" s="45">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D222" s="45">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E222" s="45">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F222" s="45">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="G222" s="45"/>
       <x:c r="H222" s="45"/>
       <x:c r="I222" s="4"/>
@@ -9118,13 +9365,27 @@
       <x:c r="A223" s="4">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="B223" s="45"/>
-      <x:c r="C223" s="45"/>
-      <x:c r="D223" s="45"/>
-      <x:c r="E223" s="45"/>
-      <x:c r="F223" s="45"/>
-      <x:c r="G223" s="45"/>
-      <x:c r="H223" s="45"/>
+      <x:c r="B223" s="45">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C223" s="45">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D223" s="45">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E223" s="45">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F223" s="45">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G223" s="45">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H223" s="45">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="I223" s="4"/>
       <x:c r="J223" s="4"/>
       <x:c r="K223" s="5"/>
@@ -9181,11 +9442,21 @@
       <x:c r="A224" s="4">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="B224" s="45"/>
-      <x:c r="C224" s="49"/>
-      <x:c r="D224" s="45"/>
-      <x:c r="E224" s="49"/>
-      <x:c r="F224" s="49"/>
+      <x:c r="B224" s="45">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="C224" s="49">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D224" s="45">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E224" s="49">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F224" s="49">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="G224" s="49"/>
       <x:c r="H224" s="49"/>
       <x:c r="I224" s="4"/>
@@ -9244,7 +9515,9 @@
       <x:c r="A225" s="4">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="B225" s="45"/>
+      <x:c r="B225" s="45">
+        <x:v>93</x:v>
+      </x:c>
       <x:c r="C225" s="45"/>
       <x:c r="D225" s="45"/>
       <x:c r="E225" s="45"/>
@@ -10516,7 +10789,7 @@
     </x:row>
     <x:row r="246" spans="1:12" ht="13.5" customHeight="1">
       <x:c r="A246" s="43" t="s">
-        <x:v>63</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="B246" s="4"/>
       <x:c r="C246" s="4"/>
@@ -10533,16 +10806,16 @@
     <x:row r="247" spans="1:12" ht="13.5" customHeight="1">
       <x:c r="A247" s="4"/>
       <x:c r="B247" s="4" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="C247" s="4" t="s">
         <x:v>51</x:v>
       </x:c>
-      <x:c r="C247" s="4" t="s">
+      <x:c r="D247" s="4" t="s">
         <x:v>52</x:v>
       </x:c>
-      <x:c r="D247" s="4" t="s">
+      <x:c r="E247" s="4" t="s">
         <x:v>53</x:v>
-      </x:c>
-      <x:c r="E247" s="4" t="s">
-        <x:v>54</x:v>
       </x:c>
       <x:c r="F247" s="4"/>
       <x:c r="G247" s="4"/>
@@ -11810,7 +12083,7 @@
     </x:row>
     <x:row r="267" spans="1:12" ht="13.5" customHeight="1">
       <x:c r="A267" s="43" t="s">
-        <x:v>64</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="B267" s="4"/>
       <x:c r="C267" s="4"/>
@@ -11827,16 +12100,16 @@
     <x:row r="268" spans="1:12" ht="13.5" customHeight="1">
       <x:c r="A268" s="4"/>
       <x:c r="B268" s="4" t="s">
-        <x:v>65</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="C268" s="4" t="s">
-        <x:v>56</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="D268" s="4" t="s">
         <x:v>47</x:v>
       </x:c>
       <x:c r="E268" s="4" t="s">
-        <x:v>66</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="F268" s="4"/>
       <x:c r="G268" s="4"/>
@@ -12982,7 +13255,7 @@
     </x:row>
     <x:row r="286" spans="1:12" ht="13.5" customHeight="1">
       <x:c r="A286" s="43" t="s">
-        <x:v>67</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="B286" s="4"/>
       <x:c r="C286" s="4"/>
@@ -13002,7 +13275,7 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="C287" s="7" t="s">
-        <x:v>68</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="D287" s="4"/>
       <x:c r="E287" s="4"/>
@@ -13018,9 +13291,7 @@
       <x:c r="A288" s="4">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B288" s="47" t="s">
-        <x:v>49</x:v>
-      </x:c>
+      <x:c r="B288" s="47"/>
       <x:c r="C288" s="56"/>
       <x:c r="D288" s="4"/>
       <x:c r="E288" s="4"/>
@@ -13074,9 +13345,7 @@
       <x:c r="A289" s="4">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B289" s="47" t="s">
-        <x:v>49</x:v>
-      </x:c>
+      <x:c r="B289" s="47"/>
       <x:c r="C289" s="56"/>
       <x:c r="D289" s="4"/>
       <x:c r="E289" s="4"/>
@@ -13130,9 +13399,7 @@
       <x:c r="A290" s="4">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B290" s="47" t="s">
-        <x:v>49</x:v>
-      </x:c>
+      <x:c r="B290" s="47"/>
       <x:c r="C290" s="56"/>
       <x:c r="D290" s="4"/>
       <x:c r="E290" s="4"/>
@@ -13186,9 +13453,7 @@
       <x:c r="A291" s="4">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B291" s="47" t="s">
-        <x:v>49</x:v>
-      </x:c>
+      <x:c r="B291" s="47"/>
       <x:c r="C291" s="56"/>
       <x:c r="D291" s="4"/>
       <x:c r="E291" s="4"/>
@@ -13242,9 +13507,7 @@
       <x:c r="A292" s="4">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B292" s="47" t="s">
-        <x:v>49</x:v>
-      </x:c>
+      <x:c r="B292" s="47"/>
       <x:c r="C292" s="56"/>
       <x:c r="D292" s="4"/>
       <x:c r="E292" s="4"/>
@@ -13298,9 +13561,7 @@
       <x:c r="A293" s="4">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B293" s="47" t="s">
-        <x:v>49</x:v>
-      </x:c>
+      <x:c r="B293" s="47"/>
       <x:c r="C293" s="57"/>
       <x:c r="D293" s="4"/>
       <x:c r="E293" s="4"/>
@@ -13366,7 +13627,7 @@
     </x:row>
     <x:row r="295" spans="1:12" ht="13.5" customHeight="1">
       <x:c r="A295" s="43" t="s">
-        <x:v>69</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="B295" s="4"/>
       <x:c r="C295" s="4"/>
@@ -13383,10 +13644,10 @@
     <x:row r="296" spans="1:12" ht="13.5" customHeight="1">
       <x:c r="A296" s="4"/>
       <x:c r="B296" s="4" t="s">
-        <x:v>56</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C296" s="4" t="s">
-        <x:v>70</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="D296" s="4"/>
       <x:c r="E296" s="4"/>
@@ -13538,7 +13799,7 @@
     </x:row>
     <x:row r="302" spans="1:12" ht="13.5" customHeight="1">
       <x:c r="A302" s="43" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="B302" s="4"/>
       <x:c r="C302" s="4"/>
@@ -13570,9 +13831,7 @@
       <x:c r="A304" s="4">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B304" s="49" t="s">
-        <x:v>49</x:v>
-      </x:c>
+      <x:c r="B304" s="49"/>
       <x:c r="C304" s="45"/>
       <x:c r="D304" s="4"/>
       <x:c r="E304" s="4"/>
@@ -13597,9 +13856,7 @@
       <x:c r="A305" s="4">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B305" s="49" t="s">
-        <x:v>49</x:v>
-      </x:c>
+      <x:c r="B305" s="49"/>
       <x:c r="C305" s="45"/>
       <x:c r="D305" s="4"/>
       <x:c r="E305" s="4"/>
@@ -13624,9 +13881,7 @@
       <x:c r="A306" s="4">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B306" s="49" t="s">
-        <x:v>49</x:v>
-      </x:c>
+      <x:c r="B306" s="49"/>
       <x:c r="C306" s="49"/>
       <x:c r="D306" s="4"/>
       <x:c r="E306" s="4"/>
@@ -13651,9 +13906,7 @@
       <x:c r="A307" s="4">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B307" s="49" t="s">
-        <x:v>49</x:v>
-      </x:c>
+      <x:c r="B307" s="49"/>
       <x:c r="C307" s="49"/>
       <x:c r="D307" s="4"/>
       <x:c r="E307" s="4"/>

</xml_diff>